<commit_message>
Aplica revisão da Semana 2 (professores e gestores)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/comunidade_semana2_diagnostico.xlsx
+++ b/kobo/comunidade_semana2_diagnostico.xlsx
@@ -5582,7 +5582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C259"/>
+  <dimension ref="A1:C260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6812,17 +6812,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>intensidade</t>
+          <t>confianca</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
@@ -6834,12 +6834,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Baixa</t>
         </is>
       </c>
     </row>
@@ -6851,12 +6851,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>media</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Média</t>
         </is>
       </c>
     </row>
@@ -6868,29 +6868,29 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>nao_se_aplica</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>acesso_mat</t>
+          <t>intensidade</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>facil</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
@@ -6902,12 +6902,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>moderado</t>
+          <t>facil</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Fácil</t>
         </is>
       </c>
     </row>
@@ -6919,12 +6919,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>dificil</t>
+          <t>moderado</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Difícil</t>
+          <t>Moderado</t>
         </is>
       </c>
     </row>
@@ -6936,12 +6936,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>dificil</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Difícil</t>
         </is>
       </c>
     </row>
@@ -6953,29 +6953,29 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>part_estud</t>
+          <t>acesso_mat</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>espectadores</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Espectadores</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6987,12 +6987,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>colaboradores_pontuais</t>
+          <t>espectadores</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Colaboradores pontuais</t>
+          <t>Espectadores</t>
         </is>
       </c>
     </row>
@@ -7004,12 +7004,12 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>protagonistas_em_alguns_momentos</t>
+          <t>colaboradores_pontuais</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Protagonistas em alguns momentos</t>
+          <t>Colaboradores pontuais</t>
         </is>
       </c>
     </row>
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>protagonistas_continuos</t>
+          <t>protagonistas_em_alguns_momentos</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Protagonistas contínuos</t>
+          <t>Protagonistas em alguns momentos</t>
         </is>
       </c>
     </row>
@@ -7038,29 +7038,29 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>protagonistas_continuos</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Protagonistas contínuos</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>continuidade_proj</t>
+          <t>part_estud</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>garantida_institucionalmente</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Garantida institucionalmente</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7072,12 +7072,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>dependente_de_pessoas_especifica</t>
+          <t>garantida_institucionalmente</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dependente de pessoas específicas</t>
+          <t>Garantida institucionalmente</t>
         </is>
       </c>
     </row>
@@ -7089,12 +7089,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>incerta</t>
+          <t>dependente_de_pessoas_especifica</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Incerta</t>
+          <t>Dependente de pessoas específicas</t>
         </is>
       </c>
     </row>
@@ -7106,29 +7106,29 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>incerta</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Incerta</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>nivel_part</t>
+          <t>continuidade_proj</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>informativa</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Informativa (recebem informação)</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7140,12 +7140,12 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>consultiva</t>
+          <t>informativa</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Consultiva (são ouvidos)</t>
+          <t>Informativa (recebem informação)</t>
         </is>
       </c>
     </row>
@@ -7157,12 +7157,12 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>colaborativa</t>
+          <t>consultiva</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Colaborativa (constroem junto)</t>
+          <t>Consultiva (são ouvidos)</t>
         </is>
       </c>
     </row>
@@ -7174,12 +7174,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>protagonista</t>
+          <t>colaborativa</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Protagonista (decidem e conduzem)</t>
+          <t>Colaborativa (constroem junto)</t>
         </is>
       </c>
     </row>
@@ -7191,29 +7191,29 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>protagonista</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Protagonista (decidem e conduzem)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>env_fam</t>
+          <t>nivel_part</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ausente</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7225,12 +7225,12 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>esporadico</t>
+          <t>ausente</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Esporádico</t>
+          <t>Ausente</t>
         </is>
       </c>
     </row>
@@ -7242,12 +7242,12 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>esporadico</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Esporádico</t>
         </is>
       </c>
     </row>
@@ -7259,12 +7259,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>ativo_protagonista</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Ativo/protagonista</t>
+          <t>Regular</t>
         </is>
       </c>
     </row>
@@ -7276,29 +7276,29 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>ativo_protagonista</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Ativo/protagonista</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>barr_fam</t>
+          <t>env_fam</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>horario_de_trabalho</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Horário de trabalho</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7310,12 +7310,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>distancia</t>
+          <t>horario_de_trabalho</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Distância</t>
+          <t>Horário de trabalho</t>
         </is>
       </c>
     </row>
@@ -7327,12 +7327,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>comunicacao_inadequada</t>
+          <t>distancia</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Comunicação inadequada</t>
+          <t>Distância</t>
         </is>
       </c>
     </row>
@@ -7344,12 +7344,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>falta_de_convite_convocacao</t>
+          <t>comunicacao_inadequada</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Falta de convite/convocação</t>
+          <t>Comunicação inadequada</t>
         </is>
       </c>
     </row>
@@ -7361,29 +7361,29 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>falta_de_convite_convocacao</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Falta de convite/convocação</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>cat_ator</t>
+          <t>barr_fam</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>sec_educacao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Secretaria de Educação</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -7395,12 +7395,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>sec_meio_amb</t>
+          <t>sec_educacao</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Secretaria de Meio Ambiente</t>
+          <t>Secretaria de Educação</t>
         </is>
       </c>
     </row>
@@ -7412,12 +7412,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>defesa_civil</t>
+          <t>sec_meio_amb</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Defesa Civil</t>
+          <t>Secretaria de Meio Ambiente</t>
         </is>
       </c>
     </row>
@@ -7429,12 +7429,12 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>sec_saude</t>
+          <t>defesa_civil</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Secretaria de Saúde</t>
+          <t>Defesa Civil</t>
         </is>
       </c>
     </row>
@@ -7446,12 +7446,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>assist_social</t>
+          <t>sec_saude</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Assistência Social</t>
+          <t>Secretaria de Saúde</t>
         </is>
       </c>
     </row>
@@ -7463,12 +7463,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>obras</t>
+          <t>assist_social</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Assistência Social</t>
         </is>
       </c>
     </row>
@@ -7480,12 +7480,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>bombeiros</t>
+          <t>obras</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Bombeiros</t>
+          <t>Obras</t>
         </is>
       </c>
     </row>
@@ -7497,12 +7497,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>ubs</t>
+          <t>bombeiros</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Bombeiros</t>
         </is>
       </c>
     </row>
@@ -7514,12 +7514,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>vigilancia</t>
+          <t>ubs</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Vigilância</t>
+          <t>UBS</t>
         </is>
       </c>
     </row>
@@ -7531,12 +7531,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>outro_publico</t>
+          <t>vigilancia</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Outro (poder público)</t>
+          <t>Vigilância</t>
         </is>
       </c>
     </row>
@@ -7548,12 +7548,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>universidade</t>
+          <t>outro_publico</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Universidade</t>
+          <t>Outro (poder público)</t>
         </is>
       </c>
     </row>
@@ -7565,12 +7565,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>inst_federal</t>
+          <t>universidade</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Instituto Federal</t>
+          <t>Universidade</t>
         </is>
       </c>
     </row>
@@ -7582,12 +7582,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>escola_tecnica</t>
+          <t>inst_federal</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Escola técnica</t>
+          <t>Instituto Federal</t>
         </is>
       </c>
     </row>
@@ -7599,12 +7599,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>centro_pesquisa</t>
+          <t>escola_tecnica</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Centro de pesquisa</t>
+          <t>Escola técnica</t>
         </is>
       </c>
     </row>
@@ -7616,12 +7616,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>museu</t>
+          <t>centro_pesquisa</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Museu</t>
+          <t>Centro de pesquisa</t>
         </is>
       </c>
     </row>
@@ -7633,12 +7633,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>jardim_botanico</t>
+          <t>museu</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Jardim botânico</t>
+          <t>Museu</t>
         </is>
       </c>
     </row>
@@ -7650,12 +7650,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>outro_educ_ciencia</t>
+          <t>jardim_botanico</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Outro (educação/ciência)</t>
+          <t>Jardim botânico</t>
         </is>
       </c>
     </row>
@@ -7667,12 +7667,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>assoc_moradores</t>
+          <t>outro_educ_ciencia</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Outro (educação/ciência)</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7684,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>ong</t>
+          <t>assoc_moradores</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>ONG</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -7701,12 +7701,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>cooperativa</t>
+          <t>ong</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>ONG</t>
         </is>
       </c>
     </row>
@@ -7718,12 +7718,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>catadores</t>
+          <t>cooperativa</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Catadores</t>
+          <t>Cooperativa</t>
         </is>
       </c>
     </row>
@@ -7735,12 +7735,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>mov_sociais</t>
+          <t>catadores</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Movimentos sociais</t>
+          <t>Catadores</t>
         </is>
       </c>
     </row>
@@ -7752,12 +7752,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>coletivos</t>
+          <t>mov_sociais</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Coletivos</t>
+          <t>Movimentos sociais</t>
         </is>
       </c>
     </row>
@@ -7769,12 +7769,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>grupos_culturais</t>
+          <t>coletivos</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Grupos culturais</t>
+          <t>Coletivos</t>
         </is>
       </c>
     </row>
@@ -7786,12 +7786,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>org_comunit_relig</t>
+          <t>grupos_culturais</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Organizações comunitárias/religiosas</t>
+          <t>Grupos culturais</t>
         </is>
       </c>
     </row>
@@ -7803,12 +7803,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>outro_soc_civil</t>
+          <t>org_comunit_relig</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Outro (sociedade civil)</t>
+          <t>Organizações comunitárias/religiosas</t>
         </is>
       </c>
     </row>
@@ -7820,12 +7820,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>povos_indigenas</t>
+          <t>outro_soc_civil</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Povos indígenas</t>
+          <t>Outro (sociedade civil)</t>
         </is>
       </c>
     </row>
@@ -7837,12 +7837,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>quilombolas</t>
+          <t>povos_indigenas</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Quilombolas</t>
+          <t>Povos indígenas</t>
         </is>
       </c>
     </row>
@@ -7854,12 +7854,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>agric_familiares</t>
+          <t>quilombolas</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Agricultores familiares</t>
+          <t>Quilombolas</t>
         </is>
       </c>
     </row>
@@ -7871,12 +7871,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>pescadores</t>
+          <t>agric_familiares</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Pescadores</t>
+          <t>Agricultores familiares</t>
         </is>
       </c>
     </row>
@@ -7888,12 +7888,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>com_tradicionais</t>
+          <t>pescadores</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Comunidades tradicionais</t>
+          <t>Pescadores</t>
         </is>
       </c>
     </row>
@@ -7905,12 +7905,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>liderancas</t>
+          <t>com_tradicionais</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Lideranças</t>
+          <t>Comunidades tradicionais</t>
         </is>
       </c>
     </row>
@@ -7922,12 +7922,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>detentores_saberes</t>
+          <t>liderancas</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Detentores de conhecimentos locais</t>
+          <t>Lideranças</t>
         </is>
       </c>
     </row>
@@ -7939,29 +7939,29 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>outro_comunidades</t>
+          <t>detentores_saberes</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Outro (comunidades e conhecimentos)</t>
+          <t>Detentores de conhecimentos locais</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>nivel_rel_grade</t>
+          <t>cat_ator</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>nao_existe</t>
+          <t>outro_comunidades</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Não existe no território</t>
+          <t>Outro (comunidades e conhecimentos)</t>
         </is>
       </c>
     </row>
@@ -7973,12 +7973,12 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>nao_sei</t>
+          <t>nao_existe</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Não sei se existe</t>
+          <t>Não existe no território</t>
         </is>
       </c>
     </row>
@@ -7990,12 +7990,12 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>sem_contato</t>
+          <t>nao_sei</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Existe, mas nunca houve contato</t>
+          <t>Não sei se existe</t>
         </is>
       </c>
     </row>
@@ -8007,12 +8007,12 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>contato_pontual</t>
+          <t>sem_contato</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Contato pontual, sem combinação formal (ainda não é parceiro(a))</t>
+          <t>Existe, mas nunca houve contato</t>
         </is>
       </c>
     </row>
@@ -8024,12 +8024,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>parceria</t>
+          <t>contato_pontual</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Parceria — já colaboram em ações combinadas</t>
+          <t>Contato pontual, sem combinação formal (ainda não é parceiro(a))</t>
         </is>
       </c>
     </row>
@@ -8041,29 +8041,29 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>articulacao</t>
+          <t>parceria</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Articulação permanente — parceria contínua e estruturada</t>
+          <t>Parceria — já colaboram em ações combinadas</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>articulacao</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Articulação permanente — parceria contínua e estruturada</t>
         </is>
       </c>
     </row>
@@ -8075,12 +8075,12 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>comunicados_impressos</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Comunicados impressos</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
@@ -8092,12 +8092,12 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>reunioes</t>
+          <t>comunicados_impressos</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Reuniões</t>
+          <t>Comunicados impressos</t>
         </is>
       </c>
     </row>
@@ -8109,12 +8109,12 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>redes_sociais</t>
+          <t>reunioes</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Redes sociais</t>
+          <t>Reuniões</t>
         </is>
       </c>
     </row>
@@ -8126,12 +8126,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>alto_falante_radio_local</t>
+          <t>redes_sociais</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Alto-falante/rádio local</t>
+          <t>Redes sociais</t>
         </is>
       </c>
     </row>
@@ -8143,29 +8143,29 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>alto_falante_radio_local</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Alto-falante/rádio local</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8177,12 +8177,12 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>parcialmente</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Parcialmente</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
@@ -8194,12 +8194,12 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>parcialmente</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Parcialmente</t>
         </is>
       </c>
     </row>
@@ -8211,29 +8211,29 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>falta_de_contato</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Falta de contato</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -8245,12 +8245,12 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>burocracia</t>
+          <t>falta_de_contato</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Burocracia</t>
+          <t>Falta de contato</t>
         </is>
       </c>
     </row>
@@ -8262,12 +8262,12 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>desconfianca_historico_de_relaca</t>
+          <t>burocracia</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Desconfiança/histórico de relação</t>
+          <t>Burocracia</t>
         </is>
       </c>
     </row>
@@ -8279,12 +8279,12 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>falta_de_tempo</t>
+          <t>desconfianca_historico_de_relaca</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Falta de tempo</t>
+          <t>Desconfiança/histórico de relação</t>
         </is>
       </c>
     </row>
@@ -8296,29 +8296,29 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>perfil_com</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>estudante</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Estudante</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -8330,12 +8330,12 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>ex_escola</t>
+          <t>estudante</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Pessoa que já trabalhou em escola, mas atualmente não trabalha</t>
+          <t>Estudante</t>
         </is>
       </c>
     </row>
@@ -8347,12 +8347,12 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>ong</t>
+          <t>ex_escola</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Pessoa de ONG ou outra organização da sociedade civil</t>
+          <t>Pessoa que já trabalhou em escola, mas atualmente não trabalha</t>
         </is>
       </c>
     </row>
@@ -8364,29 +8364,29 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>ong</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Pessoa de ONG ou outra organização da sociedade civil</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>onde_ea_com</t>
+          <t>perfil_com</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>escolas_do_territorio</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Escolas do território</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8398,12 +8398,12 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>associacoes_ongs</t>
+          <t>escolas_do_territorio</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Associações / ONGs</t>
+          <t>Escolas do território</t>
         </is>
       </c>
     </row>
@@ -8415,12 +8415,12 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>mutiroes_e_acoes_comunitarias</t>
+          <t>associacoes_ongs</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Mutirões e ações comunitárias</t>
+          <t>Associações / ONGs</t>
         </is>
       </c>
     </row>
@@ -8432,12 +8432,12 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>igrejas_grupos_religiosos</t>
+          <t>mutiroes_e_acoes_comunitarias</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Igrejas / grupos religiosos</t>
+          <t>Mutirões e ações comunitárias</t>
         </is>
       </c>
     </row>
@@ -8449,12 +8449,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>coletivos_e_grupos_de_jovens</t>
+          <t>igrejas_grupos_religiosos</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Coletivos e grupos de jovens</t>
+          <t>Igrejas / grupos religiosos</t>
         </is>
       </c>
     </row>
@@ -8466,12 +8466,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>universidades_institutos</t>
+          <t>coletivos_e_grupos_de_jovens</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Universidades / institutos</t>
+          <t>Coletivos e grupos de jovens</t>
         </is>
       </c>
     </row>
@@ -8483,12 +8483,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>rodas_de_conversa_e_oficinas</t>
+          <t>universidades_institutos</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Rodas de conversa e oficinas</t>
+          <t>Universidades / institutos</t>
         </is>
       </c>
     </row>
@@ -8500,12 +8500,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>redes_sociais_comunicacao</t>
+          <t>rodas_de_conversa_e_oficinas</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Redes sociais / comunicação</t>
+          <t>Rodas de conversa e oficinas</t>
         </is>
       </c>
     </row>
@@ -8517,12 +8517,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>nao_acontece</t>
+          <t>redes_sociais_comunicacao</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Não acontece</t>
+          <t>Redes sociais / comunicação</t>
         </is>
       </c>
     </row>
@@ -8534,29 +8534,29 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>nao_acontece</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Não acontece</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>instit_com</t>
+          <t>onde_ea_com</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8568,12 +8568,12 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>isolada_ocasional</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Isolada/ocasional</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
@@ -8585,12 +8585,12 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>recorrente_dependente_de_poucas_</t>
+          <t>isolada_ocasional</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Recorrente, dependente de poucas pessoas</t>
+          <t>Isolada/ocasional</t>
         </is>
       </c>
     </row>
@@ -8602,12 +8602,12 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>presente_em_diferentes_grupos_or</t>
+          <t>recorrente_dependente_de_poucas_</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Presente em diferentes grupos/organizações</t>
+          <t>Recorrente, dependente de poucas pessoas</t>
         </is>
       </c>
     </row>
@@ -8619,12 +8619,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>integrada_as_acoes_da_comunidade</t>
+          <t>presente_em_diferentes_grupos_or</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Integrada às ações da comunidade</t>
+          <t>Presente em diferentes grupos/organizações</t>
         </is>
       </c>
     </row>
@@ -8636,12 +8636,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>continua_e_reconhecida_pela_comu</t>
+          <t>integrada_as_acoes_da_comunidade</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Contínua e reconhecida pela comunidade</t>
+          <t>Integrada às ações da comunidade</t>
         </is>
       </c>
     </row>
@@ -8653,29 +8653,29 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>continua_e_reconhecida_pela_comu</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Contínua e reconhecida pela comunidade</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>esc_territorio</t>
+          <t>instit_com</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>sim_com_frequencia</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Sim, com frequência</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -8687,12 +8687,12 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>as_vezes</t>
+          <t>sim_com_frequencia</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Às vezes</t>
+          <t>Sim, com frequência</t>
         </is>
       </c>
     </row>
@@ -8704,12 +8704,12 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>raramente</t>
+          <t>as_vezes</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Raramente</t>
+          <t>Às vezes</t>
         </is>
       </c>
     </row>
@@ -8721,12 +8721,12 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>raramente</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Raramente</t>
         </is>
       </c>
     </row>
@@ -8738,12 +8738,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>nao_existe_escola_no_territorio</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Não existe escola no território</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
@@ -8755,29 +8755,29 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>nao_sei</t>
+          <t>nao_existe_escola_no_territorio</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Não sei</t>
+          <t>Não existe escola no território</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>contexto_ea_com</t>
+          <t>esc_territorio</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>escola</t>
+          <t>nao_sei</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Escola</t>
+          <t>Não sei</t>
         </is>
       </c>
     </row>
@@ -8789,12 +8789,12 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>espaco_comunitario_associacao</t>
+          <t>escola</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Espaço comunitário / associação</t>
+          <t>Escola</t>
         </is>
       </c>
     </row>
@@ -8806,12 +8806,12 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>rua_praca_ou_area_externa</t>
+          <t>espaco_comunitario_associacao</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Rua, praça ou área externa</t>
+          <t>Espaço comunitário / associação</t>
         </is>
       </c>
     </row>
@@ -8823,12 +8823,12 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>visita_de_campo_trilha</t>
+          <t>rua_praca_ou_area_externa</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Visita de campo / trilha</t>
+          <t>Rua, praça ou área externa</t>
         </is>
       </c>
     </row>
@@ -8840,12 +8840,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>evento_feira</t>
+          <t>visita_de_campo_trilha</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Evento / feira</t>
+          <t>Visita de campo / trilha</t>
         </is>
       </c>
     </row>
@@ -8857,12 +8857,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>online_redes_sociais</t>
+          <t>evento_feira</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Online / redes sociais</t>
+          <t>Evento / feira</t>
         </is>
       </c>
     </row>
@@ -8874,29 +8874,29 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>online_redes_sociais</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Online / redes sociais</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>quem_planejou_com</t>
+          <t>contexto_ea_com</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8908,12 +8908,12 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -8925,12 +8925,12 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>associacao_ong</t>
+          <t>professores</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Associação / ONG</t>
+          <t>Professores(as)</t>
         </is>
       </c>
     </row>
@@ -8942,12 +8942,12 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>liderancas_comunitarias</t>
+          <t>associacao_ong</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Lideranças comunitárias</t>
+          <t>Associação / ONG</t>
         </is>
       </c>
     </row>
@@ -8959,12 +8959,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>poder_publico</t>
+          <t>liderancas_comunitarias</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Poder público</t>
+          <t>Lideranças comunitárias</t>
         </is>
       </c>
     </row>
@@ -8976,12 +8976,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>universidade_instituto</t>
+          <t>poder_publico</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Universidade / instituto</t>
+          <t>Poder público</t>
         </is>
       </c>
     </row>
@@ -8993,12 +8993,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>moradores_em_geral</t>
+          <t>universidade_instituto</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Moradores em geral</t>
+          <t>Universidade / instituto</t>
         </is>
       </c>
     </row>
@@ -9010,29 +9010,29 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>moradores_em_geral</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Moradores em geral</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>continuidade_com</t>
+          <t>quem_planejou_com</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>depende_de_pessoas_especificas</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Depende de pessoas específicas</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9044,12 +9044,12 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>garantida</t>
+          <t>depende_de_pessoas_especificas</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Tem continuidade garantida (organização ou parceria)</t>
+          <t>Depende de pessoas específicas</t>
         </is>
       </c>
     </row>
@@ -9061,12 +9061,12 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>incerta</t>
+          <t>garantida</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Incerta</t>
+          <t>Tem continuidade garantida (organização ou parceria)</t>
         </is>
       </c>
     </row>
@@ -9078,29 +9078,29 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>incerta</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Incerta</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>causa_dif_com</t>
+          <t>continuidade_com</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>falta_de_formacao</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Falta de formação</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -9112,12 +9112,12 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>falta_de_material</t>
+          <t>falta_de_formacao</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Falta de material</t>
+          <t>Falta de formação</t>
         </is>
       </c>
     </row>
@@ -9129,12 +9129,12 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>tema_sensivel_delicado</t>
+          <t>falta_de_material</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Tema sensível/delicado</t>
+          <t>Falta de material</t>
         </is>
       </c>
     </row>
@@ -9146,12 +9146,12 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>falta_de_tempo</t>
+          <t>tema_sensivel_delicado</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Falta de tempo</t>
+          <t>Tema sensível/delicado</t>
         </is>
       </c>
     </row>
@@ -9163,12 +9163,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>falta_de_apoio_ou_recursos</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Falta de apoio ou recursos</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
@@ -9180,29 +9180,29 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>falta_de_apoio_ou_recursos</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Falta de apoio ou recursos</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>apoio_com</t>
+          <t>causa_dif_com</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9214,12 +9214,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>material_educativo</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Material educativo</t>
+          <t>Formação</t>
         </is>
       </c>
     </row>
@@ -9231,12 +9231,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>tempo_para_se_organizar</t>
+          <t>material_educativo</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Tempo para se organizar</t>
+          <t>Material educativo</t>
         </is>
       </c>
     </row>
@@ -9248,12 +9248,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>apoio_de_liderancas_poder_public</t>
+          <t>tempo_para_se_organizar</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Apoio de lideranças / poder público</t>
+          <t>Tempo para se organizar</t>
         </is>
       </c>
     </row>
@@ -9265,12 +9265,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>parcerias</t>
+          <t>apoio_de_liderancas_poder_public</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Parcerias</t>
+          <t>Apoio de lideranças / poder público</t>
         </is>
       </c>
     </row>
@@ -9282,12 +9282,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>recursos_financeiros</t>
+          <t>parcerias</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Recursos financeiros</t>
+          <t>Parcerias</t>
         </is>
       </c>
     </row>
@@ -9299,29 +9299,29 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>recursos_financeiros</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Recursos financeiros</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>barreiras_com</t>
+          <t>apoio_com</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>tempo</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Tempo</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9333,12 +9333,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>tempo</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Tempo</t>
         </is>
       </c>
     </row>
@@ -9350,12 +9350,12 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>materiais</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Materiais</t>
+          <t>Formação</t>
         </is>
       </c>
     </row>
@@ -9367,12 +9367,12 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>recursos_financeiros</t>
+          <t>materiais</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Recursos financeiros</t>
+          <t>Materiais</t>
         </is>
       </c>
     </row>
@@ -9384,12 +9384,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>apoio_do_poder_publico</t>
+          <t>recursos_financeiros</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Apoio do poder público</t>
+          <t>Recursos financeiros</t>
         </is>
       </c>
     </row>
@@ -9401,12 +9401,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>apoio_de_liderancas</t>
+          <t>apoio_do_poder_publico</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Apoio de lideranças</t>
+          <t>Apoio do poder público</t>
         </is>
       </c>
     </row>
@@ -9418,12 +9418,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>organizacao_coletiva_planejament</t>
+          <t>apoio_de_liderancas</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Organização coletiva / planejamento conjunto</t>
+          <t>Apoio de lideranças</t>
         </is>
       </c>
     </row>
@@ -9435,12 +9435,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>informacoes_sobre_o_territorio</t>
+          <t>organizacao_coletiva_planejament</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Informações sobre o território</t>
+          <t>Organização coletiva / planejamento conjunto</t>
         </is>
       </c>
     </row>
@@ -9452,12 +9452,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>descontinuidade_das_acoes</t>
+          <t>informacoes_sobre_o_territorio</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Descontinuidade das ações</t>
+          <t>Informações sobre o território</t>
         </is>
       </c>
     </row>
@@ -9469,12 +9469,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>rotatividade_de_pessoas</t>
+          <t>descontinuidade_das_acoes</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Rotatividade de pessoas</t>
+          <t>Descontinuidade das ações</t>
         </is>
       </c>
     </row>
@@ -9486,29 +9486,29 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>rotatividade_de_pessoas</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Rotatividade de pessoas</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>materiais_com</t>
+          <t>barreiras_com</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>livros_e_cartilhas</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Livros e cartilhas</t>
+          <t>Outras</t>
         </is>
       </c>
     </row>
@@ -9520,12 +9520,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>videos</t>
+          <t>livros_e_cartilhas</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Vídeos</t>
+          <t>Livros e cartilhas</t>
         </is>
       </c>
     </row>
@@ -9537,12 +9537,12 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>jogos</t>
+          <t>videos</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Jogos</t>
+          <t>Vídeos</t>
         </is>
       </c>
     </row>
@@ -9554,12 +9554,12 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>materiais_produzidos_pela_comuni</t>
+          <t>jogos</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Materiais produzidos pela comunidade/organização</t>
+          <t>Jogos</t>
         </is>
       </c>
     </row>
@@ -9571,12 +9571,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>recursos_digitais</t>
+          <t>materiais_produzidos_pela_comuni</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Recursos digitais</t>
+          <t>Materiais produzidos pela comunidade/organização</t>
         </is>
       </c>
     </row>
@@ -9588,12 +9588,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>recursos_digitais</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Recursos digitais</t>
         </is>
       </c>
     </row>
@@ -9605,29 +9605,29 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>quem_part_com</t>
+          <t>materiais_com</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9639,12 +9639,12 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -9656,12 +9656,12 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>familias</t>
+          <t>professores</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Famílias</t>
+          <t>Professores(as)</t>
         </is>
       </c>
     </row>
@@ -9673,12 +9673,12 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>moradores</t>
+          <t>familias</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Moradores</t>
+          <t>Famílias</t>
         </is>
       </c>
     </row>
@@ -9690,12 +9690,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>liderancas_comunitarias</t>
+          <t>moradores</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Lideranças comunitárias</t>
+          <t>Moradores</t>
         </is>
       </c>
     </row>
@@ -9707,12 +9707,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>associacoes_ongs</t>
+          <t>liderancas_comunitarias</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Associações / ONGs</t>
+          <t>Lideranças comunitárias</t>
         </is>
       </c>
     </row>
@@ -9724,12 +9724,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>poder_publico</t>
+          <t>associacoes_ongs</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Poder público</t>
+          <t>Associações / ONGs</t>
         </is>
       </c>
     </row>
@@ -9741,29 +9741,29 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>poder_publico</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Poder público</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>esp_com</t>
+          <t>quem_part_com</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>associacao_de_moradores</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
@@ -9775,12 +9775,12 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>conselho_comunitario</t>
+          <t>associacao_de_moradores</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Conselho comunitário</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -9792,12 +9792,12 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>assembleias_reunioes_comunitaria</t>
+          <t>conselho_comunitario</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Assembleias / reuniões comunitárias</t>
+          <t>Conselho comunitário</t>
         </is>
       </c>
     </row>
@@ -9809,12 +9809,12 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>gremio_estudantil_coletivos_de_j</t>
+          <t>assembleias_reunioes_comunitaria</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Grêmio estudantil / coletivos de jovens</t>
+          <t>Assembleias / reuniões comunitárias</t>
         </is>
       </c>
     </row>
@@ -9826,12 +9826,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>conselhos_de_politicas_publicas</t>
+          <t>gremio_estudantil_coletivos_de_j</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Conselhos de políticas públicas</t>
+          <t>Grêmio estudantil / coletivos de jovens</t>
         </is>
       </c>
     </row>
@@ -9843,12 +9843,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>conselhos_de_politicas_publicas</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Conselhos de políticas públicas</t>
         </is>
       </c>
     </row>
@@ -9860,29 +9860,29 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>instancias_com</t>
+          <t>esp_com</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>associacao_de_moradores</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9894,12 +9894,12 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>conselho_comunitario</t>
+          <t>associacao_de_moradores</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Conselho comunitário</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -9911,12 +9911,12 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>conselho_escolar</t>
+          <t>conselho_comunitario</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Conselho escolar</t>
+          <t>Conselho comunitário</t>
         </is>
       </c>
     </row>
@@ -9928,12 +9928,12 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>conselhos_de_politicas_publicas</t>
+          <t>conselho_escolar</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Conselhos de políticas públicas</t>
+          <t>Conselho escolar</t>
         </is>
       </c>
     </row>
@@ -9945,12 +9945,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>gremio_coletivos</t>
+          <t>conselhos_de_politicas_publicas</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Grêmio / coletivos</t>
+          <t>Conselhos de políticas públicas</t>
         </is>
       </c>
     </row>
@@ -9962,12 +9962,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>nenhuma</t>
+          <t>gremio_coletivos</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Grêmio / coletivos</t>
         </is>
       </c>
     </row>
@@ -9979,10 +9979,27 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
+          <t>nenhuma</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>instancias_com</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
           <t>outro</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr">
+      <c r="C260" t="inlineStr">
         <is>
           <t>Outra</t>
         </is>

</xml_diff>

<commit_message>
Semana 2: adiciona opção Não sabe em Q2.6, Q2.9, Q2.22, Q2.24, Q2.25 e Q2.37
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/comunidade_semana2_diagnostico.xlsx
+++ b/kobo/comunidade_semana2_diagnostico.xlsx
@@ -995,8 +995,16 @@
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>not(selected(., 'nao_sabe') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>"Não sabe" não pode ser combinado com outras opções.</t>
+        </is>
+      </c>
       <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
@@ -1071,8 +1079,16 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>not(selected(., 'nao_sabe') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>"Não sabe" não pode ser combinado com outras opções.</t>
+        </is>
+      </c>
       <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
@@ -1911,8 +1927,16 @@
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>not(selected(., 'nao_sabe') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>"Não sabe" não pode ser combinado com outras opções.</t>
+        </is>
+      </c>
       <c r="J57" t="inlineStr"/>
     </row>
     <row r="58">
@@ -2023,8 +2047,16 @@
       <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>not(selected(., 'nao_sabe') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>"Não sabe" não pode ser combinado com outras opções.</t>
+        </is>
+      </c>
       <c r="J61" t="inlineStr"/>
     </row>
     <row r="62">
@@ -2803,8 +2835,16 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
       <c r="G91" t="inlineStr"/>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr"/>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>not(selected(., 'nao_sabe') and count-selected(.) &gt; 1)</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>"Não sabe" não pode ser combinado com outras opções.</t>
+        </is>
+      </c>
       <c r="J91" t="inlineStr"/>
     </row>
     <row r="92">
@@ -5582,7 +5622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C260"/>
+  <dimension ref="A1:C263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5945,17 +5985,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>freq_ea</t>
+          <t>areas_curr</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>diaria</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Diária</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -5967,12 +6007,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>semanal</t>
+          <t>diaria</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Semanal</t>
+          <t>Diária</t>
         </is>
       </c>
     </row>
@@ -5984,12 +6024,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>mensal</t>
+          <t>semanal</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mensal</t>
+          <t>Semanal</t>
         </is>
       </c>
     </row>
@@ -6001,12 +6041,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>esporadica</t>
+          <t>mensal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Esporádica</t>
+          <t>Mensal</t>
         </is>
       </c>
     </row>
@@ -6018,12 +6058,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>anual</t>
+          <t>esporadica</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Anual</t>
+          <t>Esporádica</t>
         </is>
       </c>
     </row>
@@ -6035,12 +6075,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>nao_ocorre</t>
+          <t>anual</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Não ocorre</t>
+          <t>Anual</t>
         </is>
       </c>
     </row>
@@ -6052,29 +6092,29 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>nao_ocorre</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Não ocorre</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>papel_estud</t>
+          <t>freq_ea</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>espectador</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Espectador</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6086,12 +6126,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>participante_pontual</t>
+          <t>espectador</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Participante pontual</t>
+          <t>Espectador</t>
         </is>
       </c>
     </row>
@@ -6103,12 +6143,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>protagonista</t>
+          <t>participante_pontual</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Protagonista</t>
+          <t>Participante pontual</t>
         </is>
       </c>
     </row>
@@ -6120,12 +6160,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>coprodutor</t>
+          <t>protagonista</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Coprodutor</t>
+          <t>Protagonista</t>
         </is>
       </c>
     </row>
@@ -6137,29 +6177,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>coprodutor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Coprodutor</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>freq5</t>
+          <t>papel_estud</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>nunca</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nunca</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6171,12 +6211,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>raramente</t>
+          <t>nunca</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Raramente</t>
+          <t>Nunca</t>
         </is>
       </c>
     </row>
@@ -6188,12 +6228,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>as_vezes</t>
+          <t>raramente</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Às vezes</t>
+          <t>Raramente</t>
         </is>
       </c>
     </row>
@@ -6205,12 +6245,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>frequentemente</t>
+          <t>as_vezes</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Frequentemente</t>
+          <t>Às vezes</t>
         </is>
       </c>
     </row>
@@ -6222,29 +6262,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>frequentemente</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Frequentemente</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>temas</t>
+          <t>freq5</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>agua</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Água</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6256,12 +6296,12 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>biodiversidade</t>
+          <t>agua</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Biodiversidade</t>
+          <t>Água</t>
         </is>
       </c>
     </row>
@@ -6273,12 +6313,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>residuos</t>
+          <t>biodiversidade</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Resíduos</t>
+          <t>Biodiversidade</t>
         </is>
       </c>
     </row>
@@ -6290,12 +6330,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>mudancas_climaticas</t>
+          <t>residuos</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Mudanças climáticas</t>
+          <t>Resíduos</t>
         </is>
       </c>
     </row>
@@ -6307,12 +6347,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>energia</t>
+          <t>mudancas_climaticas</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Energia</t>
+          <t>Mudanças climáticas</t>
         </is>
       </c>
     </row>
@@ -6324,12 +6364,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>alimentacao</t>
+          <t>energia</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Alimentação</t>
+          <t>Energia</t>
         </is>
       </c>
     </row>
@@ -6341,12 +6381,12 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>consumo</t>
+          <t>alimentacao</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Consumo</t>
+          <t>Alimentação</t>
         </is>
       </c>
     </row>
@@ -6358,12 +6398,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>saneamento</t>
+          <t>consumo</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Saneamento</t>
+          <t>Consumo</t>
         </is>
       </c>
     </row>
@@ -6375,12 +6415,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>saude</t>
+          <t>saneamento</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Saúde</t>
+          <t>Saneamento</t>
         </is>
       </c>
     </row>
@@ -6392,12 +6432,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>riscos_desastres</t>
+          <t>saude</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Riscos/desastres</t>
+          <t>Saúde</t>
         </is>
       </c>
     </row>
@@ -6409,12 +6449,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>justica_socioambiental</t>
+          <t>riscos_desastres</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Justiça socioambiental</t>
+          <t>Riscos/desastres</t>
         </is>
       </c>
     </row>
@@ -6426,12 +6466,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>territorio</t>
+          <t>justica_socioambiental</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Território</t>
+          <t>Justiça socioambiental</t>
         </is>
       </c>
     </row>
@@ -6443,12 +6483,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>conflitos</t>
+          <t>territorio</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Conflitos</t>
+          <t>Território</t>
         </is>
       </c>
     </row>
@@ -6460,12 +6500,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>povos_e_comunidades_tradicionais</t>
+          <t>conflitos</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Povos e comunidades tradicionais</t>
+          <t>Conflitos</t>
         </is>
       </c>
     </row>
@@ -6477,46 +6517,46 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>povos_e_comunidades_tradicionais</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Povos e comunidades tradicionais</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>metodos</t>
+          <t>temas</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>aula_expositiva</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Aula expositiva</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>metodos</t>
+          <t>temas</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>projeto</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Projeto</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6528,12 +6568,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>oficina</t>
+          <t>aula_expositiva</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Oficina</t>
+          <t>Aula expositiva</t>
         </is>
       </c>
     </row>
@@ -6545,12 +6585,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>saida_de_campo</t>
+          <t>projeto</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Saída de campo</t>
+          <t>Projeto</t>
         </is>
       </c>
     </row>
@@ -6562,12 +6602,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>horta_experimentacao</t>
+          <t>oficina</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Horta/experimentação</t>
+          <t>Oficina</t>
         </is>
       </c>
     </row>
@@ -6579,12 +6619,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>rodas_de_conversa</t>
+          <t>saida_de_campo</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Rodas de conversa</t>
+          <t>Saída de campo</t>
         </is>
       </c>
     </row>
@@ -6596,12 +6636,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>producao_audiovisual</t>
+          <t>horta_experimentacao</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Produção audiovisual</t>
+          <t>Horta/experimentação</t>
         </is>
       </c>
     </row>
@@ -6613,12 +6653,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>cartografia</t>
+          <t>rodas_de_conversa</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cartografia</t>
+          <t>Rodas de conversa</t>
         </is>
       </c>
     </row>
@@ -6630,63 +6670,63 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>producao_audiovisual</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Produção audiovisual</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>impacto_form</t>
+          <t>metodos</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>cartografia</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Cartografia</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>impacto_form</t>
+          <t>metodos</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>pouco</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pouco</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>impacto_form</t>
+          <t>metodos</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>moderado</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6698,12 +6738,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>significativo</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Significativo</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
@@ -6715,63 +6755,63 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>pouco</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Pouco</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>confianca</t>
+          <t>impacto_form</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>moderado</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>1 — Nada confiante(a)</t>
+          <t>Moderado</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>confianca</t>
+          <t>impacto_form</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>significativo</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2 — Pouco confiante</t>
+          <t>Significativo</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>confianca</t>
+          <t>impacto_form</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>3 — Moderadamente confiante</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -6783,12 +6823,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>4 — Confiante</t>
+          <t>1 — Nada confiante(a)</t>
         </is>
       </c>
     </row>
@@ -6800,12 +6840,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>5 — Muito confiante</t>
+          <t>2 — Pouco confiante</t>
         </is>
       </c>
     </row>
@@ -6817,63 +6857,63 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>nao_se_aplica</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>3 — Moderadamente confiante</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>intensidade</t>
+          <t>confianca</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>4 — Confiante</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>intensidade</t>
+          <t>confianca</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>5 — Muito confiante</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>intensidade</t>
+          <t>confianca</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
@@ -6885,63 +6925,63 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>nao_se_aplica</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Não se aplica</t>
+          <t>Baixa</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>acesso_mat</t>
+          <t>intensidade</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>facil</t>
+          <t>media</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Fácil</t>
+          <t>Média</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>acesso_mat</t>
+          <t>intensidade</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>moderado</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Moderado</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>acesso_mat</t>
+          <t>intensidade</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>dificil</t>
+          <t>nao_se_aplica</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Difícil</t>
+          <t>Não se aplica</t>
         </is>
       </c>
     </row>
@@ -6953,12 +6993,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>facil</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Fácil</t>
         </is>
       </c>
     </row>
@@ -6970,63 +7010,63 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>moderado</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Moderado</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>part_estud</t>
+          <t>acesso_mat</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>espectadores</t>
+          <t>dificil</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Espectadores</t>
+          <t>Difícil</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>part_estud</t>
+          <t>acesso_mat</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>colaboradores_pontuais</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Colaboradores pontuais</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>part_estud</t>
+          <t>acesso_mat</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>protagonistas_em_alguns_momentos</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Protagonistas em alguns momentos</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7038,12 +7078,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>protagonistas_continuos</t>
+          <t>espectadores</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Protagonistas contínuos</t>
+          <t>Espectadores</t>
         </is>
       </c>
     </row>
@@ -7055,63 +7095,63 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>colaboradores_pontuais</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Colaboradores pontuais</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>continuidade_proj</t>
+          <t>part_estud</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>garantida_institucionalmente</t>
+          <t>protagonistas_em_alguns_momentos</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Garantida institucionalmente</t>
+          <t>Protagonistas em alguns momentos</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>continuidade_proj</t>
+          <t>part_estud</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>dependente_de_pessoas_especifica</t>
+          <t>protagonistas_continuos</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Dependente de pessoas específicas</t>
+          <t>Protagonistas contínuos</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>continuidade_proj</t>
+          <t>part_estud</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>incerta</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Incerta</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7123,63 +7163,63 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>garantida_institucionalmente</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Garantida institucionalmente</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>nivel_part</t>
+          <t>continuidade_proj</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>informativa</t>
+          <t>dependente_de_pessoas_especifica</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Informativa (recebem informação)</t>
+          <t>Dependente de pessoas específicas</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>nivel_part</t>
+          <t>continuidade_proj</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>consultiva</t>
+          <t>incerta</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Consultiva (são ouvidos)</t>
+          <t>Incerta</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>nivel_part</t>
+          <t>continuidade_proj</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>colaborativa</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Colaborativa (constroem junto)</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7191,12 +7231,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>protagonista</t>
+          <t>informativa</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Protagonista (decidem e conduzem)</t>
+          <t>Informativa (recebem informação)</t>
         </is>
       </c>
     </row>
@@ -7208,63 +7248,63 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>consultiva</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Consultiva (são ouvidos)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>env_fam</t>
+          <t>nivel_part</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>ausente</t>
+          <t>colaborativa</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Ausente</t>
+          <t>Colaborativa (constroem junto)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>env_fam</t>
+          <t>nivel_part</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>esporadico</t>
+          <t>protagonista</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Esporádico</t>
+          <t>Protagonista (decidem e conduzem)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>env_fam</t>
+          <t>nivel_part</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7276,12 +7316,12 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>ativo_protagonista</t>
+          <t>ausente</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Ativo/protagonista</t>
+          <t>Ausente</t>
         </is>
       </c>
     </row>
@@ -7293,63 +7333,63 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>esporadico</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Esporádico</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>barr_fam</t>
+          <t>env_fam</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>horario_de_trabalho</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Horário de trabalho</t>
+          <t>Regular</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>barr_fam</t>
+          <t>env_fam</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>distancia</t>
+          <t>ativo_protagonista</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Distância</t>
+          <t>Ativo/protagonista</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>barr_fam</t>
+          <t>env_fam</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>comunicacao_inadequada</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Comunicação inadequada</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -7361,12 +7401,12 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>falta_de_convite_convocacao</t>
+          <t>horario_de_trabalho</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Falta de convite/convocação</t>
+          <t>Horário de trabalho</t>
         </is>
       </c>
     </row>
@@ -7378,63 +7418,63 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>distancia</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Distância</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>cat_ator</t>
+          <t>barr_fam</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>sec_educacao</t>
+          <t>comunicacao_inadequada</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Secretaria de Educação</t>
+          <t>Comunicação inadequada</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>cat_ator</t>
+          <t>barr_fam</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>sec_meio_amb</t>
+          <t>falta_de_convite_convocacao</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Secretaria de Meio Ambiente</t>
+          <t>Falta de convite/convocação</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>cat_ator</t>
+          <t>barr_fam</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>defesa_civil</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Defesa Civil</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -7446,12 +7486,12 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>sec_saude</t>
+          <t>sec_educacao</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Secretaria de Saúde</t>
+          <t>Secretaria de Educação</t>
         </is>
       </c>
     </row>
@@ -7463,12 +7503,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>assist_social</t>
+          <t>sec_meio_amb</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Assistência Social</t>
+          <t>Secretaria de Meio Ambiente</t>
         </is>
       </c>
     </row>
@@ -7480,12 +7520,12 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>obras</t>
+          <t>defesa_civil</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Obras</t>
+          <t>Defesa Civil</t>
         </is>
       </c>
     </row>
@@ -7497,12 +7537,12 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>bombeiros</t>
+          <t>sec_saude</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Bombeiros</t>
+          <t>Secretaria de Saúde</t>
         </is>
       </c>
     </row>
@@ -7514,12 +7554,12 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>ubs</t>
+          <t>assist_social</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>UBS</t>
+          <t>Assistência Social</t>
         </is>
       </c>
     </row>
@@ -7531,12 +7571,12 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>vigilancia</t>
+          <t>obras</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Vigilância</t>
+          <t>Obras</t>
         </is>
       </c>
     </row>
@@ -7548,12 +7588,12 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>outro_publico</t>
+          <t>bombeiros</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Outro (poder público)</t>
+          <t>Bombeiros</t>
         </is>
       </c>
     </row>
@@ -7565,12 +7605,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>universidade</t>
+          <t>ubs</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Universidade</t>
+          <t>UBS</t>
         </is>
       </c>
     </row>
@@ -7582,12 +7622,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>inst_federal</t>
+          <t>vigilancia</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Instituto Federal</t>
+          <t>Vigilância</t>
         </is>
       </c>
     </row>
@@ -7599,12 +7639,12 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>escola_tecnica</t>
+          <t>outro_publico</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Escola técnica</t>
+          <t>Outro (poder público)</t>
         </is>
       </c>
     </row>
@@ -7616,12 +7656,12 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>centro_pesquisa</t>
+          <t>universidade</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Centro de pesquisa</t>
+          <t>Universidade</t>
         </is>
       </c>
     </row>
@@ -7633,12 +7673,12 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>museu</t>
+          <t>inst_federal</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Museu</t>
+          <t>Instituto Federal</t>
         </is>
       </c>
     </row>
@@ -7650,12 +7690,12 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>jardim_botanico</t>
+          <t>escola_tecnica</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Jardim botânico</t>
+          <t>Escola técnica</t>
         </is>
       </c>
     </row>
@@ -7667,12 +7707,12 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>outro_educ_ciencia</t>
+          <t>centro_pesquisa</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Outro (educação/ciência)</t>
+          <t>Centro de pesquisa</t>
         </is>
       </c>
     </row>
@@ -7684,12 +7724,12 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>assoc_moradores</t>
+          <t>museu</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Museu</t>
         </is>
       </c>
     </row>
@@ -7701,12 +7741,12 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>ong</t>
+          <t>jardim_botanico</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>ONG</t>
+          <t>Jardim botânico</t>
         </is>
       </c>
     </row>
@@ -7718,12 +7758,12 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>cooperativa</t>
+          <t>outro_educ_ciencia</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Cooperativa</t>
+          <t>Outro (educação/ciência)</t>
         </is>
       </c>
     </row>
@@ -7735,12 +7775,12 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>catadores</t>
+          <t>assoc_moradores</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Catadores</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -7752,12 +7792,12 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>mov_sociais</t>
+          <t>ong</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Movimentos sociais</t>
+          <t>ONG</t>
         </is>
       </c>
     </row>
@@ -7769,12 +7809,12 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>coletivos</t>
+          <t>cooperativa</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Coletivos</t>
+          <t>Cooperativa</t>
         </is>
       </c>
     </row>
@@ -7786,12 +7826,12 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>grupos_culturais</t>
+          <t>catadores</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Grupos culturais</t>
+          <t>Catadores</t>
         </is>
       </c>
     </row>
@@ -7803,12 +7843,12 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>org_comunit_relig</t>
+          <t>mov_sociais</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Organizações comunitárias/religiosas</t>
+          <t>Movimentos sociais</t>
         </is>
       </c>
     </row>
@@ -7820,12 +7860,12 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>outro_soc_civil</t>
+          <t>coletivos</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Outro (sociedade civil)</t>
+          <t>Coletivos</t>
         </is>
       </c>
     </row>
@@ -7837,12 +7877,12 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>povos_indigenas</t>
+          <t>grupos_culturais</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Povos indígenas</t>
+          <t>Grupos culturais</t>
         </is>
       </c>
     </row>
@@ -7854,12 +7894,12 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>quilombolas</t>
+          <t>org_comunit_relig</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>Quilombolas</t>
+          <t>Organizações comunitárias/religiosas</t>
         </is>
       </c>
     </row>
@@ -7871,12 +7911,12 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>agric_familiares</t>
+          <t>outro_soc_civil</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Agricultores familiares</t>
+          <t>Outro (sociedade civil)</t>
         </is>
       </c>
     </row>
@@ -7888,12 +7928,12 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>pescadores</t>
+          <t>povos_indigenas</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Pescadores</t>
+          <t>Povos indígenas</t>
         </is>
       </c>
     </row>
@@ -7905,12 +7945,12 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>com_tradicionais</t>
+          <t>quilombolas</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Comunidades tradicionais</t>
+          <t>Quilombolas</t>
         </is>
       </c>
     </row>
@@ -7922,12 +7962,12 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>liderancas</t>
+          <t>agric_familiares</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Lideranças</t>
+          <t>Agricultores familiares</t>
         </is>
       </c>
     </row>
@@ -7939,12 +7979,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>detentores_saberes</t>
+          <t>pescadores</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Detentores de conhecimentos locais</t>
+          <t>Pescadores</t>
         </is>
       </c>
     </row>
@@ -7956,63 +7996,63 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>outro_comunidades</t>
+          <t>com_tradicionais</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Outro (comunidades e conhecimentos)</t>
+          <t>Comunidades tradicionais</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>nivel_rel_grade</t>
+          <t>cat_ator</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>nao_existe</t>
+          <t>liderancas</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Não existe no território</t>
+          <t>Lideranças</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>nivel_rel_grade</t>
+          <t>cat_ator</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>nao_sei</t>
+          <t>detentores_saberes</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Não sei se existe</t>
+          <t>Detentores de conhecimentos locais</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>nivel_rel_grade</t>
+          <t>cat_ator</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>sem_contato</t>
+          <t>outro_comunidades</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Existe, mas nunca houve contato</t>
+          <t>Outro (comunidades e conhecimentos)</t>
         </is>
       </c>
     </row>
@@ -8024,12 +8064,12 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>contato_pontual</t>
+          <t>nao_existe</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Contato pontual, sem combinação formal (ainda não é parceiro(a))</t>
+          <t>Não existe no território</t>
         </is>
       </c>
     </row>
@@ -8041,12 +8081,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>parceria</t>
+          <t>nao_sei</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Parceria — já colaboram em ações combinadas</t>
+          <t>Não sei se existe</t>
         </is>
       </c>
     </row>
@@ -8058,63 +8098,63 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>articulacao</t>
+          <t>sem_contato</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Articulação permanente — parceria contínua e estruturada</t>
+          <t>Existe, mas nunca houve contato</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>whatsapp</t>
+          <t>contato_pontual</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>WhatsApp</t>
+          <t>Contato pontual, sem combinação formal (ainda não é parceiro(a))</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>comunicados_impressos</t>
+          <t>parceria</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Comunicados impressos</t>
+          <t>Parceria — já colaboram em ações combinadas</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>canais</t>
+          <t>nivel_rel_grade</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>reunioes</t>
+          <t>articulacao</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Reuniões</t>
+          <t>Articulação permanente — parceria contínua e estruturada</t>
         </is>
       </c>
     </row>
@@ -8126,12 +8166,12 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>redes_sociais</t>
+          <t>whatsapp</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Redes sociais</t>
+          <t>WhatsApp</t>
         </is>
       </c>
     </row>
@@ -8143,12 +8183,12 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>alto_falante_radio_local</t>
+          <t>comunicados_impressos</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Alto-falante/rádio local</t>
+          <t>Comunicados impressos</t>
         </is>
       </c>
     </row>
@@ -8160,63 +8200,63 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>reunioes</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Reuniões</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>redes_sociais</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Redes sociais</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>parcialmente</t>
+          <t>alto_falante_radio_local</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Parcialmente</t>
+          <t>Alto-falante/rádio local</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>suficiente</t>
+          <t>canais</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8228,63 +8268,63 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>falta_de_contato</t>
+          <t>parcialmente</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Falta de contato</t>
+          <t>Parcialmente</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>burocracia</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Burocracia</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>barr_artic</t>
+          <t>suficiente</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>desconfianca_historico_de_relaca</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Desconfiança/histórico de relação</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -8296,12 +8336,12 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>falta_de_tempo</t>
+          <t>falta_de_contato</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Falta de tempo</t>
+          <t>Falta de contato</t>
         </is>
       </c>
     </row>
@@ -8313,63 +8353,63 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>burocracia</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Burocracia</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>perfil_com</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>estudante</t>
+          <t>desconfianca_historico_de_relaca</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Estudante</t>
+          <t>Desconfiança/histórico de relação</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>perfil_com</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>ex_escola</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Pessoa que já trabalhou em escola, mas atualmente não trabalha</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>perfil_com</t>
+          <t>barr_artic</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ong</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Pessoa de ONG ou outra organização da sociedade civil</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -8381,63 +8421,63 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>estudante</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Estudante</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>onde_ea_com</t>
+          <t>perfil_com</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>escolas_do_territorio</t>
+          <t>ex_escola</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Escolas do território</t>
+          <t>Pessoa que já trabalhou em escola, mas atualmente não trabalha</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>onde_ea_com</t>
+          <t>perfil_com</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>associacoes_ongs</t>
+          <t>ong</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Associações / ONGs</t>
+          <t>Pessoa de ONG ou outra organização da sociedade civil</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>onde_ea_com</t>
+          <t>perfil_com</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>mutiroes_e_acoes_comunitarias</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Mutirões e ações comunitárias</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8449,12 +8489,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>igrejas_grupos_religiosos</t>
+          <t>escolas_do_territorio</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Igrejas / grupos religiosos</t>
+          <t>Escolas do território</t>
         </is>
       </c>
     </row>
@@ -8466,12 +8506,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>coletivos_e_grupos_de_jovens</t>
+          <t>associacoes_ongs</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Coletivos e grupos de jovens</t>
+          <t>Associações / ONGs</t>
         </is>
       </c>
     </row>
@@ -8483,12 +8523,12 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>universidades_institutos</t>
+          <t>mutiroes_e_acoes_comunitarias</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Universidades / institutos</t>
+          <t>Mutirões e ações comunitárias</t>
         </is>
       </c>
     </row>
@@ -8500,12 +8540,12 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>rodas_de_conversa_e_oficinas</t>
+          <t>igrejas_grupos_religiosos</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Rodas de conversa e oficinas</t>
+          <t>Igrejas / grupos religiosos</t>
         </is>
       </c>
     </row>
@@ -8517,12 +8557,12 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>redes_sociais_comunicacao</t>
+          <t>coletivos_e_grupos_de_jovens</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Redes sociais / comunicação</t>
+          <t>Coletivos e grupos de jovens</t>
         </is>
       </c>
     </row>
@@ -8534,12 +8574,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>nao_acontece</t>
+          <t>universidades_institutos</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Não acontece</t>
+          <t>Universidades / institutos</t>
         </is>
       </c>
     </row>
@@ -8551,63 +8591,63 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>rodas_de_conversa_e_oficinas</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Rodas de conversa e oficinas</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>instit_com</t>
+          <t>onde_ea_com</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>redes_sociais_comunicacao</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Redes sociais / comunicação</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>instit_com</t>
+          <t>onde_ea_com</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>isolada_ocasional</t>
+          <t>nao_acontece</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Isolada/ocasional</t>
+          <t>Não acontece</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>instit_com</t>
+          <t>onde_ea_com</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>recorrente_dependente_de_poucas_</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Recorrente, dependente de poucas pessoas</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8619,12 +8659,12 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>presente_em_diferentes_grupos_or</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Presente em diferentes grupos/organizações</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
@@ -8636,12 +8676,12 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>integrada_as_acoes_da_comunidade</t>
+          <t>isolada_ocasional</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Integrada às ações da comunidade</t>
+          <t>Isolada/ocasional</t>
         </is>
       </c>
     </row>
@@ -8653,12 +8693,12 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>continua_e_reconhecida_pela_comu</t>
+          <t>recorrente_dependente_de_poucas_</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Contínua e reconhecida pela comunidade</t>
+          <t>Recorrente, dependente de poucas pessoas</t>
         </is>
       </c>
     </row>
@@ -8670,63 +8710,63 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>presente_em_diferentes_grupos_or</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Presente em diferentes grupos/organizações</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>esc_territorio</t>
+          <t>instit_com</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>sim_com_frequencia</t>
+          <t>integrada_as_acoes_da_comunidade</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Sim, com frequência</t>
+          <t>Integrada às ações da comunidade</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>esc_territorio</t>
+          <t>instit_com</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>as_vezes</t>
+          <t>continua_e_reconhecida_pela_comu</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Às vezes</t>
+          <t>Contínua e reconhecida pela comunidade</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>esc_territorio</t>
+          <t>instit_com</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>raramente</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Raramente</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -8738,12 +8778,12 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>sim_com_frequencia</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim, com frequência</t>
         </is>
       </c>
     </row>
@@ -8755,12 +8795,12 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>nao_existe_escola_no_territorio</t>
+          <t>as_vezes</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Não existe escola no território</t>
+          <t>Às vezes</t>
         </is>
       </c>
     </row>
@@ -8772,63 +8812,63 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>nao_sei</t>
+          <t>raramente</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Não sei</t>
+          <t>Raramente</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>contexto_ea_com</t>
+          <t>esc_territorio</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>escola</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Escola</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>contexto_ea_com</t>
+          <t>esc_territorio</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>espaco_comunitario_associacao</t>
+          <t>nao_existe_escola_no_territorio</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Espaço comunitário / associação</t>
+          <t>Não existe escola no território</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>contexto_ea_com</t>
+          <t>esc_territorio</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>rua_praca_ou_area_externa</t>
+          <t>nao_sei</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Rua, praça ou área externa</t>
+          <t>Não sei</t>
         </is>
       </c>
     </row>
@@ -8840,12 +8880,12 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>visita_de_campo_trilha</t>
+          <t>escola</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Visita de campo / trilha</t>
+          <t>Escola</t>
         </is>
       </c>
     </row>
@@ -8857,12 +8897,12 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>evento_feira</t>
+          <t>espaco_comunitario_associacao</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Evento / feira</t>
+          <t>Espaço comunitário / associação</t>
         </is>
       </c>
     </row>
@@ -8874,12 +8914,12 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>online_redes_sociais</t>
+          <t>rua_praca_ou_area_externa</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>Online / redes sociais</t>
+          <t>Rua, praça ou área externa</t>
         </is>
       </c>
     </row>
@@ -8891,63 +8931,63 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>visita_de_campo_trilha</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Visita de campo / trilha</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>quem_planejou_com</t>
+          <t>contexto_ea_com</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>evento_feira</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Evento / feira</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>quem_planejou_com</t>
+          <t>contexto_ea_com</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>online_redes_sociais</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Online / redes sociais</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>quem_planejou_com</t>
+          <t>contexto_ea_com</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>associacao_ong</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Associação / ONG</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -8959,12 +8999,12 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>liderancas_comunitarias</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Lideranças comunitárias</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -8976,12 +9016,12 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>poder_publico</t>
+          <t>professores</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Poder público</t>
+          <t>Professores(as)</t>
         </is>
       </c>
     </row>
@@ -8993,12 +9033,12 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>universidade_instituto</t>
+          <t>associacao_ong</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Universidade / instituto</t>
+          <t>Associação / ONG</t>
         </is>
       </c>
     </row>
@@ -9010,12 +9050,12 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>moradores_em_geral</t>
+          <t>liderancas_comunitarias</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Moradores em geral</t>
+          <t>Lideranças comunitárias</t>
         </is>
       </c>
     </row>
@@ -9027,63 +9067,63 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>poder_publico</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Poder público</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>continuidade_com</t>
+          <t>quem_planejou_com</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>depende_de_pessoas_especificas</t>
+          <t>universidade_instituto</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Depende de pessoas específicas</t>
+          <t>Universidade / instituto</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>continuidade_com</t>
+          <t>quem_planejou_com</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>garantida</t>
+          <t>moradores_em_geral</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Tem continuidade garantida (organização ou parceria)</t>
+          <t>Moradores em geral</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>continuidade_com</t>
+          <t>quem_planejou_com</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>incerta</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Incerta</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9095,63 +9135,63 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>depende_de_pessoas_especificas</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Depende de pessoas específicas</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>causa_dif_com</t>
+          <t>continuidade_com</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>falta_de_formacao</t>
+          <t>garantida</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Falta de formação</t>
+          <t>Tem continuidade garantida (organização ou parceria)</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>causa_dif_com</t>
+          <t>continuidade_com</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>falta_de_material</t>
+          <t>incerta</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Falta de material</t>
+          <t>Incerta</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>causa_dif_com</t>
+          <t>continuidade_com</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>tema_sensivel_delicado</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Tema sensível/delicado</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -9163,12 +9203,12 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>falta_de_tempo</t>
+          <t>falta_de_formacao</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Falta de tempo</t>
+          <t>Falta de formação</t>
         </is>
       </c>
     </row>
@@ -9180,12 +9220,12 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>falta_de_apoio_ou_recursos</t>
+          <t>falta_de_material</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Falta de apoio ou recursos</t>
+          <t>Falta de material</t>
         </is>
       </c>
     </row>
@@ -9197,63 +9237,63 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>tema_sensivel_delicado</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Tema sensível/delicado</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>apoio_com</t>
+          <t>causa_dif_com</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>falta_de_tempo</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Falta de tempo</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>apoio_com</t>
+          <t>causa_dif_com</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>material_educativo</t>
+          <t>falta_de_apoio_ou_recursos</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Material educativo</t>
+          <t>Falta de apoio ou recursos</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>apoio_com</t>
+          <t>causa_dif_com</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>tempo_para_se_organizar</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Tempo para se organizar</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9265,12 +9305,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>apoio_de_liderancas_poder_public</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Apoio de lideranças / poder público</t>
+          <t>Formação</t>
         </is>
       </c>
     </row>
@@ -9282,12 +9322,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>parcerias</t>
+          <t>material_educativo</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Parcerias</t>
+          <t>Material educativo</t>
         </is>
       </c>
     </row>
@@ -9299,12 +9339,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>recursos_financeiros</t>
+          <t>tempo_para_se_organizar</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Recursos financeiros</t>
+          <t>Tempo para se organizar</t>
         </is>
       </c>
     </row>
@@ -9316,63 +9356,63 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>apoio_de_liderancas_poder_public</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Apoio de lideranças / poder público</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>barreiras_com</t>
+          <t>apoio_com</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>tempo</t>
+          <t>parcerias</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Tempo</t>
+          <t>Parcerias</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>barreiras_com</t>
+          <t>apoio_com</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>formacao</t>
+          <t>recursos_financeiros</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Recursos financeiros</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>barreiras_com</t>
+          <t>apoio_com</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>materiais</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Materiais</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9384,12 +9424,12 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>recursos_financeiros</t>
+          <t>tempo</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>Recursos financeiros</t>
+          <t>Tempo</t>
         </is>
       </c>
     </row>
@@ -9401,12 +9441,12 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>apoio_do_poder_publico</t>
+          <t>formacao</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Apoio do poder público</t>
+          <t>Formação</t>
         </is>
       </c>
     </row>
@@ -9418,12 +9458,12 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>apoio_de_liderancas</t>
+          <t>materiais</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Apoio de lideranças</t>
+          <t>Materiais</t>
         </is>
       </c>
     </row>
@@ -9435,12 +9475,12 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>organizacao_coletiva_planejament</t>
+          <t>recursos_financeiros</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Organização coletiva / planejamento conjunto</t>
+          <t>Recursos financeiros</t>
         </is>
       </c>
     </row>
@@ -9452,12 +9492,12 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>informacoes_sobre_o_territorio</t>
+          <t>apoio_do_poder_publico</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Informações sobre o território</t>
+          <t>Apoio do poder público</t>
         </is>
       </c>
     </row>
@@ -9469,12 +9509,12 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>descontinuidade_das_acoes</t>
+          <t>apoio_de_liderancas</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Descontinuidade das ações</t>
+          <t>Apoio de lideranças</t>
         </is>
       </c>
     </row>
@@ -9486,12 +9526,12 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>rotatividade_de_pessoas</t>
+          <t>organizacao_coletiva_planejament</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Rotatividade de pessoas</t>
+          <t>Organização coletiva / planejamento conjunto</t>
         </is>
       </c>
     </row>
@@ -9503,63 +9543,63 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>informacoes_sobre_o_territorio</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Outras</t>
+          <t>Informações sobre o território</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>materiais_com</t>
+          <t>barreiras_com</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>livros_e_cartilhas</t>
+          <t>descontinuidade_das_acoes</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Livros e cartilhas</t>
+          <t>Descontinuidade das ações</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>materiais_com</t>
+          <t>barreiras_com</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>videos</t>
+          <t>rotatividade_de_pessoas</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Vídeos</t>
+          <t>Rotatividade de pessoas</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>materiais_com</t>
+          <t>barreiras_com</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>jogos</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Jogos</t>
+          <t>Outras</t>
         </is>
       </c>
     </row>
@@ -9571,12 +9611,12 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>materiais_produzidos_pela_comuni</t>
+          <t>livros_e_cartilhas</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>Materiais produzidos pela comunidade/organização</t>
+          <t>Livros e cartilhas</t>
         </is>
       </c>
     </row>
@@ -9588,12 +9628,12 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>recursos_digitais</t>
+          <t>videos</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>Recursos digitais</t>
+          <t>Vídeos</t>
         </is>
       </c>
     </row>
@@ -9605,12 +9645,12 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>jogos</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Jogos</t>
         </is>
       </c>
     </row>
@@ -9622,63 +9662,63 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>materiais_produzidos_pela_comuni</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Materiais produzidos pela comunidade/organização</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>quem_part_com</t>
+          <t>materiais_com</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>recursos_digitais</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Recursos digitais</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>quem_part_com</t>
+          <t>materiais_com</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>quem_part_com</t>
+          <t>materiais_com</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>familias</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Famílias</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9690,12 +9730,12 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>moradores</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Moradores</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -9707,12 +9747,12 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>liderancas_comunitarias</t>
+          <t>professores</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Lideranças comunitárias</t>
+          <t>Professores(as)</t>
         </is>
       </c>
     </row>
@@ -9724,12 +9764,12 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>associacoes_ongs</t>
+          <t>familias</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Associações / ONGs</t>
+          <t>Famílias</t>
         </is>
       </c>
     </row>
@@ -9741,12 +9781,12 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>poder_publico</t>
+          <t>moradores</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Poder público</t>
+          <t>Moradores</t>
         </is>
       </c>
     </row>
@@ -9758,63 +9798,63 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>liderancas_comunitarias</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Lideranças comunitárias</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>esp_com</t>
+          <t>quem_part_com</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>associacao_de_moradores</t>
+          <t>associacoes_ongs</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Associações / ONGs</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>esp_com</t>
+          <t>quem_part_com</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>conselho_comunitario</t>
+          <t>poder_publico</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Conselho comunitário</t>
+          <t>Poder público</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>esp_com</t>
+          <t>quem_part_com</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>assembleias_reunioes_comunitaria</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Assembleias / reuniões comunitárias</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
@@ -9826,12 +9866,12 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>gremio_estudantil_coletivos_de_j</t>
+          <t>associacao_de_moradores</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Grêmio estudantil / coletivos de jovens</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -9843,12 +9883,12 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>conselhos_de_politicas_publicas</t>
+          <t>conselho_comunitario</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Conselhos de políticas públicas</t>
+          <t>Conselho comunitário</t>
         </is>
       </c>
     </row>
@@ -9860,12 +9900,12 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>assembleias_reunioes_comunitaria</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Assembleias / reuniões comunitárias</t>
         </is>
       </c>
     </row>
@@ -9877,63 +9917,63 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>gremio_estudantil_coletivos_de_j</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Grêmio estudantil / coletivos de jovens</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>instancias_com</t>
+          <t>esp_com</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>associacao_de_moradores</t>
+          <t>conselhos_de_politicas_publicas</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Associação de moradores</t>
+          <t>Conselhos de políticas públicas</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>instancias_com</t>
+          <t>esp_com</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>conselho_comunitario</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Conselho comunitário</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>instancias_com</t>
+          <t>esp_com</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>conselho_escolar</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Conselho escolar</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -9945,12 +9985,12 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>conselhos_de_politicas_publicas</t>
+          <t>associacao_de_moradores</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Conselhos de políticas públicas</t>
+          <t>Associação de moradores</t>
         </is>
       </c>
     </row>
@@ -9962,12 +10002,12 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>gremio_coletivos</t>
+          <t>conselho_comunitario</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Grêmio / coletivos</t>
+          <t>Conselho comunitário</t>
         </is>
       </c>
     </row>
@@ -9979,12 +10019,12 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>nenhuma</t>
+          <t>conselho_escolar</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Nenhuma</t>
+          <t>Conselho escolar</t>
         </is>
       </c>
     </row>
@@ -9996,10 +10036,61 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
+          <t>conselhos_de_politicas_publicas</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Conselhos de políticas públicas</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>instancias_com</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>gremio_coletivos</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Grêmio / coletivos</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>instancias_com</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>nenhuma</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Nenhuma</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>instancias_com</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
           <t>outro</t>
         </is>
       </c>
-      <c r="C260" t="inlineStr">
+      <c r="C263" t="inlineStr">
         <is>
           <t>Outra</t>
         </is>

</xml_diff>